<commit_message>
fix(carton): complete historical imports and warehouse launch workflows
</commit_message>
<xml_diff>
--- a/public/templates/carton-history-inventory-import-template.xlsx
+++ b/public/templates/carton-history-inventory-import-template.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="期初库存导入" sheetId="1" r:id="Rfb55446b86314b2c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写示例" sheetId="2" r:id="R81ea42d7b0414ee9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="3" r:id="R70d6f7e22fe74719"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="期初库存导入" sheetId="1" r:id="R5d83af78c56a4e2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写示例" sheetId="2" r:id="Rd28f17bf197846ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="3" r:id="Rc1e6b3bad66c462c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15,12 +15,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="3">
+  <x:numFmts count="4">
     <x:numFmt numFmtId="200" formatCode="@"/>
     <x:numFmt numFmtId="201" formatCode="General"/>
     <x:numFmt numFmtId="202" formatCode="0.00"/>
+    <x:numFmt numFmtId="203" formatCode="yyyy-mm-dd hh:mm"/>
   </x:numFmts>
-  <x:fonts count="7">
+  <x:fonts count="8">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -59,8 +60,14 @@
       <x:color rgb="FF1F3F5B"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="14">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -97,6 +104,36 @@
         <x:fgColor rgb="FFF4F7FB"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF64748B"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF4F7FB"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF64748B"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF4F7FB"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="4">
     <x:border/>
@@ -122,7 +159,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="57">
+  <x:cellXfs count="69">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -289,6 +326,28 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -550,6 +609,8 @@
     <x:col min="11" max="11" width="25" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="38" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="22" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="16" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="26" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
@@ -614,6 +675,12 @@
       </x:c>
       <x:c r="M2" s="9" t="str">
         <x:v>原结余金额</x:v>
+      </x:c>
+      <x:c r="N2" s="64" t="str">
+        <x:v>仓库</x:v>
+      </x:c>
+      <x:c r="O2" s="68" t="str">
+        <x:v>入库时间</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="30" customHeight="1">
@@ -630,6 +697,8 @@
       <x:c r="K3" s="36"/>
       <x:c r="L3" s="21"/>
       <x:c r="M3" s="39"/>
+      <x:c r="N3" s="65" t="str"/>
+      <x:c r="O3" s="67" t="str"/>
     </x:row>
     <x:row r="4" ht="30" customHeight="1">
       <x:c r="A4" s="19"/>
@@ -645,6 +714,8 @@
       <x:c r="K4" s="37"/>
       <x:c r="L4" s="22"/>
       <x:c r="M4" s="40"/>
+      <x:c r="N4" s="65" t="str"/>
+      <x:c r="O4" s="67" t="str"/>
     </x:row>
     <x:row r="5" ht="30" customHeight="1">
       <x:c r="A5" s="19"/>
@@ -660,6 +731,8 @@
       <x:c r="K5" s="37"/>
       <x:c r="L5" s="22"/>
       <x:c r="M5" s="40"/>
+      <x:c r="N5" s="65" t="str"/>
+      <x:c r="O5" s="67" t="str"/>
     </x:row>
     <x:row r="6" ht="30" customHeight="1">
       <x:c r="A6" s="19"/>
@@ -675,6 +748,8 @@
       <x:c r="K6" s="37"/>
       <x:c r="L6" s="22"/>
       <x:c r="M6" s="40"/>
+      <x:c r="N6" s="65" t="str"/>
+      <x:c r="O6" s="67" t="str"/>
     </x:row>
     <x:row r="7" ht="30" customHeight="1">
       <x:c r="A7" s="19"/>
@@ -690,6 +765,8 @@
       <x:c r="K7" s="37"/>
       <x:c r="L7" s="22"/>
       <x:c r="M7" s="40"/>
+      <x:c r="N7" s="65" t="str"/>
+      <x:c r="O7" s="67" t="str"/>
     </x:row>
     <x:row r="8" ht="30" customHeight="1">
       <x:c r="A8" s="19"/>
@@ -705,6 +782,8 @@
       <x:c r="K8" s="37"/>
       <x:c r="L8" s="22"/>
       <x:c r="M8" s="40"/>
+      <x:c r="N8" s="65" t="str"/>
+      <x:c r="O8" s="67" t="str"/>
     </x:row>
     <x:row r="9" ht="30" customHeight="1">
       <x:c r="A9" s="19"/>
@@ -720,6 +799,8 @@
       <x:c r="K9" s="37"/>
       <x:c r="L9" s="22"/>
       <x:c r="M9" s="40"/>
+      <x:c r="N9" s="65" t="str"/>
+      <x:c r="O9" s="67" t="str"/>
     </x:row>
     <x:row r="10" ht="30" customHeight="1">
       <x:c r="A10" s="19"/>
@@ -735,6 +816,8 @@
       <x:c r="K10" s="37"/>
       <x:c r="L10" s="22"/>
       <x:c r="M10" s="40"/>
+      <x:c r="N10" s="65" t="str"/>
+      <x:c r="O10" s="67" t="str"/>
     </x:row>
     <x:row r="11" ht="30" customHeight="1">
       <x:c r="A11" s="19"/>
@@ -750,6 +833,8 @@
       <x:c r="K11" s="37"/>
       <x:c r="L11" s="22"/>
       <x:c r="M11" s="40"/>
+      <x:c r="N11" s="65" t="str"/>
+      <x:c r="O11" s="67" t="str"/>
     </x:row>
     <x:row r="12" ht="30" customHeight="1">
       <x:c r="A12" s="19"/>
@@ -765,6 +850,8 @@
       <x:c r="K12" s="37"/>
       <x:c r="L12" s="22"/>
       <x:c r="M12" s="40"/>
+      <x:c r="N12" s="65" t="str"/>
+      <x:c r="O12" s="67" t="str"/>
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
       <x:c r="A13" s="19"/>
@@ -780,6 +867,8 @@
       <x:c r="K13" s="37"/>
       <x:c r="L13" s="22"/>
       <x:c r="M13" s="40"/>
+      <x:c r="N13" s="65" t="str"/>
+      <x:c r="O13" s="67" t="str"/>
     </x:row>
     <x:row r="14" ht="30" customHeight="1">
       <x:c r="A14" s="19"/>
@@ -795,6 +884,8 @@
       <x:c r="K14" s="37"/>
       <x:c r="L14" s="22"/>
       <x:c r="M14" s="40"/>
+      <x:c r="N14" s="65" t="str"/>
+      <x:c r="O14" s="67" t="str"/>
     </x:row>
     <x:row r="15" ht="30" customHeight="1">
       <x:c r="A15" s="19"/>
@@ -810,6 +901,8 @@
       <x:c r="K15" s="37"/>
       <x:c r="L15" s="22"/>
       <x:c r="M15" s="40"/>
+      <x:c r="N15" s="65" t="str"/>
+      <x:c r="O15" s="67" t="str"/>
     </x:row>
     <x:row r="16" ht="30" customHeight="1">
       <x:c r="A16" s="19"/>
@@ -825,6 +918,8 @@
       <x:c r="K16" s="37"/>
       <x:c r="L16" s="22"/>
       <x:c r="M16" s="40"/>
+      <x:c r="N16" s="65" t="str"/>
+      <x:c r="O16" s="67" t="str"/>
     </x:row>
     <x:row r="17" ht="30" customHeight="1">
       <x:c r="A17" s="19"/>
@@ -840,6 +935,8 @@
       <x:c r="K17" s="37"/>
       <x:c r="L17" s="22"/>
       <x:c r="M17" s="40"/>
+      <x:c r="N17" s="65" t="str"/>
+      <x:c r="O17" s="67" t="str"/>
     </x:row>
     <x:row r="18" ht="30" customHeight="1">
       <x:c r="A18" s="19"/>
@@ -855,6 +952,8 @@
       <x:c r="K18" s="37"/>
       <x:c r="L18" s="22"/>
       <x:c r="M18" s="40"/>
+      <x:c r="N18" s="65" t="str"/>
+      <x:c r="O18" s="67" t="str"/>
     </x:row>
     <x:row r="19" ht="30" customHeight="1">
       <x:c r="A19" s="19"/>
@@ -870,6 +969,8 @@
       <x:c r="K19" s="37"/>
       <x:c r="L19" s="22"/>
       <x:c r="M19" s="40"/>
+      <x:c r="N19" s="65" t="str"/>
+      <x:c r="O19" s="67" t="str"/>
     </x:row>
     <x:row r="20" ht="30" customHeight="1">
       <x:c r="A20" s="19"/>
@@ -885,6 +986,8 @@
       <x:c r="K20" s="37"/>
       <x:c r="L20" s="22"/>
       <x:c r="M20" s="40"/>
+      <x:c r="N20" s="65" t="str"/>
+      <x:c r="O20" s="67" t="str"/>
     </x:row>
     <x:row r="21" ht="30" customHeight="1">
       <x:c r="A21" s="19"/>
@@ -900,6 +1003,8 @@
       <x:c r="K21" s="37"/>
       <x:c r="L21" s="22"/>
       <x:c r="M21" s="40"/>
+      <x:c r="N21" s="65" t="str"/>
+      <x:c r="O21" s="67" t="str"/>
     </x:row>
     <x:row r="22" ht="30" customHeight="1">
       <x:c r="A22" s="19"/>
@@ -915,6 +1020,8 @@
       <x:c r="K22" s="37"/>
       <x:c r="L22" s="22"/>
       <x:c r="M22" s="40"/>
+      <x:c r="N22" s="65" t="str"/>
+      <x:c r="O22" s="67" t="str"/>
     </x:row>
     <x:row r="23" ht="30" customHeight="1">
       <x:c r="A23" s="19"/>
@@ -930,6 +1037,8 @@
       <x:c r="K23" s="37"/>
       <x:c r="L23" s="22"/>
       <x:c r="M23" s="40"/>
+      <x:c r="N23" s="65" t="str"/>
+      <x:c r="O23" s="67" t="str"/>
     </x:row>
     <x:row r="24" ht="30" customHeight="1">
       <x:c r="A24" s="19"/>
@@ -945,6 +1054,8 @@
       <x:c r="K24" s="37"/>
       <x:c r="L24" s="22"/>
       <x:c r="M24" s="40"/>
+      <x:c r="N24" s="65" t="str"/>
+      <x:c r="O24" s="67" t="str"/>
     </x:row>
     <x:row r="25" ht="30" customHeight="1">
       <x:c r="A25" s="19"/>
@@ -960,6 +1071,8 @@
       <x:c r="K25" s="37"/>
       <x:c r="L25" s="22"/>
       <x:c r="M25" s="40"/>
+      <x:c r="N25" s="65" t="str"/>
+      <x:c r="O25" s="67" t="str"/>
     </x:row>
     <x:row r="26" ht="30" customHeight="1">
       <x:c r="A26" s="19"/>
@@ -975,6 +1088,8 @@
       <x:c r="K26" s="37"/>
       <x:c r="L26" s="22"/>
       <x:c r="M26" s="40"/>
+      <x:c r="N26" s="65" t="str"/>
+      <x:c r="O26" s="67" t="str"/>
     </x:row>
     <x:row r="27" ht="30" customHeight="1">
       <x:c r="A27" s="19"/>
@@ -990,6 +1105,8 @@
       <x:c r="K27" s="37"/>
       <x:c r="L27" s="22"/>
       <x:c r="M27" s="40"/>
+      <x:c r="N27" s="65" t="str"/>
+      <x:c r="O27" s="67" t="str"/>
     </x:row>
     <x:row r="28" ht="30" customHeight="1">
       <x:c r="A28" s="19"/>
@@ -1005,6 +1122,8 @@
       <x:c r="K28" s="37"/>
       <x:c r="L28" s="22"/>
       <x:c r="M28" s="40"/>
+      <x:c r="N28" s="65" t="str"/>
+      <x:c r="O28" s="67" t="str"/>
     </x:row>
     <x:row r="29" ht="30" customHeight="1">
       <x:c r="A29" s="19"/>
@@ -1020,6 +1139,8 @@
       <x:c r="K29" s="37"/>
       <x:c r="L29" s="22"/>
       <x:c r="M29" s="40"/>
+      <x:c r="N29" s="65" t="str"/>
+      <x:c r="O29" s="67" t="str"/>
     </x:row>
     <x:row r="30" ht="30" customHeight="1">
       <x:c r="A30" s="19"/>
@@ -1035,6 +1156,8 @@
       <x:c r="K30" s="37"/>
       <x:c r="L30" s="22"/>
       <x:c r="M30" s="40"/>
+      <x:c r="N30" s="65" t="str"/>
+      <x:c r="O30" s="67" t="str"/>
     </x:row>
     <x:row r="31" ht="30" customHeight="1">
       <x:c r="A31" s="19"/>
@@ -1050,6 +1173,8 @@
       <x:c r="K31" s="37"/>
       <x:c r="L31" s="22"/>
       <x:c r="M31" s="40"/>
+      <x:c r="N31" s="65" t="str"/>
+      <x:c r="O31" s="67" t="str"/>
     </x:row>
     <x:row r="32" ht="30" customHeight="1">
       <x:c r="A32" s="20"/>
@@ -1065,11 +1190,13 @@
       <x:c r="K32" s="38"/>
       <x:c r="L32" s="23"/>
       <x:c r="M32" s="41"/>
+      <x:c r="N32" s="65" t="str"/>
+      <x:c r="O32" s="67" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra01a43083b0647db"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R211593821c004806"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1094,6 +1221,8 @@
     <x:col min="11" max="11" width="25" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="38" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="22" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="16" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="26" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -1130,7 +1259,7 @@
     </x:row>
     <x:row r="3" ht="32" customHeight="1">
       <x:c r="A3" s="44" t="str">
-        <x:v>演示批次：客户迪奇，仓库 A，基准日期 2026-09-01，尺寸 cm，币种 CNY。实际信息请在页面选择。</x:v>
+        <x:v>示例：客户迪奇，仓库 A，尺寸 cm，币种 CNY；入库时间按每行填写，不再另选基准日期。</x:v>
       </x:c>
       <x:c r="B3" s="44"/>
       <x:c r="C3" s="44"/>
@@ -1200,6 +1329,12 @@
       <x:c r="M5" s="9" t="str">
         <x:v>原结余金额</x:v>
       </x:c>
+      <x:c r="N5" s="64" t="str">
+        <x:v>仓库</x:v>
+      </x:c>
+      <x:c r="O5" s="68" t="str">
+        <x:v>入库时间</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="30" customHeight="1">
       <x:c r="A6" s="21" t="str">
@@ -1240,6 +1375,12 @@
       </x:c>
       <x:c r="M6" s="39" t="n">
         <x:v>250</x:v>
+      </x:c>
+      <x:c r="N6" s="65" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="O6" s="67" t="n">
+        <x:v>46254.395833333336</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="30" customHeight="1">
@@ -1274,6 +1415,12 @@
         <x:v>示例：单价未知，留空待核价</x:v>
       </x:c>
       <x:c r="M7" s="40"/>
+      <x:c r="N7" s="65" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="O7" s="67" t="n">
+        <x:v>46255</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="30" customHeight="1">
       <x:c r="A8" s="22" t="str">
@@ -1312,6 +1459,12 @@
       </x:c>
       <x:c r="M8" s="40" t="n">
         <x:v>15</x:v>
+      </x:c>
+      <x:c r="N8" s="65" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="O8" s="67" t="n">
+        <x:v>46256</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="30" customHeight="1">
@@ -1346,6 +1499,14 @@
         <x:v>示例：零结余行跳过</x:v>
       </x:c>
       <x:c r="M9" s="41"/>
+      <x:c r="N9" s="65" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="O9" s="67"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="N10" s="65" t="str"/>
+      <x:c r="O10" s="67" t="str"/>
     </x:row>
     <x:row r="11" ht="32" customHeight="1">
       <x:c r="A11" s="1" t="str">
@@ -1363,6 +1524,8 @@
       <x:c r="K11" s="1"/>
       <x:c r="L11" s="1"/>
       <x:c r="M11" s="1"/>
+      <x:c r="N11" s="65" t="str"/>
+      <x:c r="O11" s="67" t="str"/>
     </x:row>
     <x:row r="12" ht="32" customHeight="1">
       <x:c r="A12" s="1" t="str">
@@ -1380,6 +1543,8 @@
       <x:c r="K12" s="1"/>
       <x:c r="L12" s="1"/>
       <x:c r="M12" s="1"/>
+      <x:c r="N12" s="65" t="str"/>
+      <x:c r="O12" s="67" t="str"/>
     </x:row>
     <x:row r="13" ht="32" customHeight="1">
       <x:c r="A13" s="1" t="str">
@@ -1397,11 +1562,13 @@
       <x:c r="K13" s="1"/>
       <x:c r="L13" s="1"/>
       <x:c r="M13" s="1"/>
+      <x:c r="N13" s="65" t="str"/>
+      <x:c r="O13" s="67" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2cc161e5274547b8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a3d5915f1044adc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1451,10 +1618,10 @@
         <x:v>批次信息在页面选</x:v>
       </x:c>
       <x:c r="B5" s="51" t="str">
-        <x:v>选择客户、仓库、期初基准日期、尺寸单位及币种，再上传文件。</x:v>
+        <x:v>页面仅选择尺寸单位；客户和仓库可不选。</x:v>
       </x:c>
       <x:c r="C5" s="51" t="str">
-        <x:v>同一文件只放这个批次的库存。不同客户、仓库或基准日期分批处理。</x:v>
+        <x:v>入库时间在文件中逐行填写，可含多个仓库和不同日期。</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="54" customHeight="1">
@@ -1462,7 +1629,7 @@
         <x:v>从哪里开始填</x:v>
       </x:c>
       <x:c r="B6" s="52" t="str">
-        <x:v>从“期初库存导入”第3行填写。日常使用前9列，单价可留空。</x:v>
+        <x:v>从“期初库存导入”第3行填写；除纸品、结余、仓位外，须填O列入库时间。</x:v>
       </x:c>
       <x:c r="C6" s="52" t="str">
         <x:v>主表空行跳过，“填写示例”和“字段说明”不参与导入。</x:v>
@@ -1506,10 +1673,10 @@
         <x:v>仓位</x:v>
       </x:c>
       <x:c r="B10" s="52" t="str">
-        <x:v>填所选仓库中的实际仓位名称，例如 A1。</x:v>
+        <x:v>填写基础资料中已有的仓位；仓库在新增“仓库”列逐行填写。</x:v>
       </x:c>
       <x:c r="C10" s="52" t="str">
-        <x:v>仓位须匹配基础资料。不同仓位的结余分行填写。</x:v>
+        <x:v>仓位名称重复时必须填仓库；唯一仓位可自动匹配仓库。</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="54" customHeight="1">
@@ -1517,7 +1684,7 @@
         <x:v>期初库存数量</x:v>
       </x:c>
       <x:c r="B11" s="52" t="str">
-        <x:v>填基准日实际还在库的结余。零结余可填0，该行会跳过。</x:v>
+        <x:v>填写实际尚在库的结余，按本行入库时间登记；无结余填0，该行跳过。</x:v>
       </x:c>
       <x:c r="C11" s="52" t="str">
         <x:v>不是历史累计入库，也不是原订单需求。不要重复增加已在系统中的库存。</x:v>
@@ -1550,7 +1717,7 @@
         <x:v>原结余金额（选填）</x:v>
       </x:c>
       <x:c r="B14" s="52" t="str">
-        <x:v>只填与本行基准日结余对应的账面金额。</x:v>
+        <x:v>只填与本行实际结余对应的库存金额。</x:v>
       </x:c>
       <x:c r="C14" s="52" t="str">
         <x:v>用于核对结余数量×单价，不是原入库金额；缺价时不反推单价。</x:v>
@@ -1591,13 +1758,13 @@
     </x:row>
     <x:row r="18" ht="54" customHeight="1">
       <x:c r="A18" s="55" t="str">
-        <x:v>不需要抄的旧列</x:v>
+        <x:v>入库时间（必填）</x:v>
       </x:c>
       <x:c r="B18" s="52" t="str">
-        <x:v>原入库日期、累计进货、累计出库及原入库金额不用填写。</x:v>
+        <x:v>填写完整日期或时间，例如 2026-08-20 09:30；旧模板“原入库时间”列仍支持。</x:v>
       </x:c>
       <x:c r="C18" s="52" t="str">
-        <x:v>这些旧历史不会被重放成新的入库、出库或供应商账款。</x:v>
+        <x:v>按行时间归属库存月份；缺失、无年份、非法或未来日期须先修正。</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="54" customHeight="1">
@@ -1623,14 +1790,26 @@
       </x:c>
     </x:row>
     <x:row r="21" ht="30" customHeight="1">
-      <x:c r="A21" s="2"/>
-      <x:c r="B21" s="2"/>
-      <x:c r="C21" s="2"/>
+      <x:c r="A21" s="2" t="str">
+        <x:v>仓库</x:v>
+      </x:c>
+      <x:c r="B21" s="2" t="str">
+        <x:v>填写基础资料中已有的仓库名称，例如 A。</x:v>
+      </x:c>
+      <x:c r="C21" s="2" t="str">
+        <x:v>每行可填写不同仓库；与该行仓位共同匹配，不自动创建仓库。</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="30" customHeight="1">
-      <x:c r="A22" s="2"/>
-      <x:c r="B22" s="2"/>
-      <x:c r="C22" s="2"/>
+      <x:c r="A22" s="2" t="str">
+        <x:v>历史月份</x:v>
+      </x:c>
+      <x:c r="B22" s="2" t="str">
+        <x:v>原入库时间所在月或后续月份已锁账时，请由主管先核对。</x:v>
+      </x:c>
+      <x:c r="C22" s="2" t="str">
+        <x:v>导入的是当前结余，不重放历史收发，也不自动还原历史每月真实库存。</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="30" customHeight="1">
       <x:c r="A23" s="2"/>

</xml_diff>